<commit_message>
Rebuild invoice PDF to match real invoice format (issuer info, tax split, numbering, due date)
Based on an actual past invoice the user provided as a reference.
Adds fixed issuer details (company info, registration number, bank
account), auto-numbering (YYYYMM-NNN, incrementing per month via a
local counter file), and due-date calculation (last day of the month
after issue month, per the user's confirmed rule).

Extends the spreadsheet schema with per-line date and tax rate, plus
matter (件名) and delivery date (納品日) columns, and splits the
subtotal/tax by 10%/8% rate to match the reference invoice's
breakdown. Verified against the reference: A社's total matches
exactly (82,500円).
</commit_message>
<xml_diff>
--- a/invoice_agent/sample_data.xlsx
+++ b/invoice_agent/sample_data.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -46,8 +48,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,17 +427,37 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>日付</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>品目</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>数量</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>単価</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>税率</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>件名</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>納品日</t>
         </is>
       </c>
     </row>
@@ -444,16 +467,30 @@
           <t>A社</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Webサイト制作</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
+      <c r="B2" s="1" t="n">
+        <v>46219</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>MTG</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
         <v>1</v>
       </c>
-      <c r="D2" t="n">
-        <v>300000</v>
+      <c r="E2" t="n">
+        <v>75000</v>
+      </c>
+      <c r="F2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>営業（販売促進）資料作成 他</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="n">
+        <v>46230</v>
       </c>
     </row>
     <row r="3">
@@ -462,34 +499,62 @@
           <t>A社</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>サーバー保守（月額）</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
+      <c r="B3" s="1" t="n">
+        <v>46225</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>MTG（たたき台案へのすり合わせ）</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
         <v>1</v>
       </c>
-      <c r="D3" t="n">
-        <v>20000</v>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>10</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>営業（販売促進）資料作成 他</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="n">
+        <v>46230</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>B社</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>ロゴデザイン</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
+          <t>A社</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>46230</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>営業（販売促進）資料納品</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
         <v>1</v>
       </c>
-      <c r="D4" t="n">
-        <v>80000</v>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>営業（販売促進）資料作成 他</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="n">
+        <v>46230</v>
       </c>
     </row>
     <row r="5">
@@ -498,16 +563,62 @@
           <t>B社</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ロゴデザイン</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>80000</v>
+      </c>
+      <c r="F5" t="n">
+        <v>10</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>ロゴ・名刺デザイン一式</t>
+        </is>
+      </c>
+      <c r="H5" s="1" t="n">
+        <v>46223</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>B社</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>46223</v>
+      </c>
+      <c r="C6" t="inlineStr">
         <is>
           <t>名刺デザイン</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="D6" t="n">
         <v>100</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E6" t="n">
         <v>50</v>
+      </c>
+      <c r="F6" t="n">
+        <v>10</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>ロゴ・名刺デザイン一式</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="n">
+        <v>46223</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rework invoice PDF layout to visually match the reference invoice
Replaces the simple top-to-bottom cell flow with positioned blocks
mirroring the WillWay reference: top black accent bar, underlined
recipient/matter/delivery-date fields with issuer info block
positioned alongside, a prominent underlined total amount line, and
a shaded table with per-tax-rate section header rows (「●税率10%項目」
etc.) instead of a plain tax-rate column.

Bundled line items with no individual price (e.g. follow-up meeting
rows under one billed item) now render with blank qty/price/amount
cells instead of 0, matching how the reference invoice presents them.
</commit_message>
<xml_diff>
--- a/invoice_agent/sample_data.xlsx
+++ b/invoice_agent/sample_data.xlsx
@@ -507,12 +507,6 @@
           <t>MTG（たたき台案へのすり合わせ）</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
       <c r="F3" t="n">
         <v>10</v>
       </c>
@@ -538,12 +532,6 @@
         <is>
           <t>営業（販売促進）資料納品</t>
         </is>
-      </c>
-      <c r="D4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0</v>
       </c>
       <c r="F4" t="n">
         <v>10</v>

</xml_diff>